<commit_message>
Updated with new location data
</commit_message>
<xml_diff>
--- a/data-engineering/tests/Emergency_Contact_Simple_Testing_Tracker_Updated.xlsx
+++ b/data-engineering/tests/Emergency_Contact_Simple_Testing_Tracker_Updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nairs\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\surab\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337BD8D3-A814-43A6-B43C-E56B18FE44C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4E1635-4B68-4C39-942A-6D33D74CABD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Emergency Contact Tests" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
   <si>
     <t>Emergency Contact Testing Tracker</t>
   </si>
@@ -86,6 +86,33 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>VA</t>
+  </si>
+  <si>
+    <t>Ashburn</t>
+  </si>
+  <si>
+    <t>Blacksburg</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>Toronto</t>
+  </si>
+  <si>
+    <t>Ontario</t>
+  </si>
+  <si>
+    <t>ON</t>
+  </si>
+  <si>
+    <t>Canada</t>
   </si>
 </sst>
 </file>
@@ -1080,17 +1107,110 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
-      <c r="G9" s="3"/>
-      <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="G10" s="3"/>
-      <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="G11" s="3"/>
-      <c r="K11" s="3"/>
+    <row r="9" spans="1:11" ht="28.5">
+      <c r="A9" s="1">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="28.5">
+      <c r="A10" s="1">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="28.5">
+      <c r="A11" s="1">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="12" spans="1:11">
       <c r="G12" s="3"/>

</xml_diff>